<commit_message>
ci: add GitHub Actions workflow and update test cases dashboard
</commit_message>
<xml_diff>
--- a/selenium/reports/test_results.xlsx
+++ b/selenium/reports/test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E3"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -501,6 +501,1714 @@
         </is>
       </c>
     </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:00:00</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>test_TC016_dashboard_patient_greeting</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="8d4c5d55d48e0009cf91974f9a665987")&gt;
+    def test_TC016_dashboard_patient_greeting(driver):
+        """TC016: Patient dashboard greeting message and username rendering"""
+&gt;       dashb</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC016_dashboard_patient_greeting.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:00:17</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>test_TC017_last_diagnostic_card</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="9f5077dddfdfbf13d415492595fc500a")&gt;
+    def test_TC017_last_diagnostic_card(driver):
+        """TC017: Last diagnostic status card check"""
+&gt;       dashboard = login_and_get_dashboard</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC017_last_diagnostic_card.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:00:35</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>test_TC018_quick_services_presence</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="34314fe0611c6a7371ab086852404050")&gt;
+    def test_TC018_quick_services_presence(driver):
+        """TC018: Quick services links presence verification"""
+&gt;       dashboard = login_and_g</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC018_quick_services_presence.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:00:52</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>test_TC019_navigation_bottom_bar_links</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="91267eacb82d13f38ef6f4e1e4fe73bf")&gt;
+    def test_TC019_navigation_bottom_bar_links(driver):
+        """TC019: Navigation bottom bar links verification"""
+&gt;       dashboard = login_and</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC019_navigation_bottom_bar_links.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:01:11</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC020]</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="6666b0b575ce9a429976e199327fd24a")&gt;
+service_name = 'upload', expected_header = 'AI Lung Diagnosis'
+test_id = 'TC020'
+    @pytest.mark.parametrize("service_name,expected_header,test_id</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC020].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:01:27</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC021]</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="8353248be2aa94bbe39ae36e98ecb525")&gt;
+service_name = 'exercises', expected_header = 'Guided Exercises'
+test_id = 'TC021'
+    @pytest.mark.parametrize("service_name,expected_header,test_</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC021].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:01:44</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC022]</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="d96a56aad1f2111e5dff523519933e37")&gt;
+service_name = 'medication', expected_header = 'Medication Log'
+test_id = 'TC022'
+    @pytest.mark.parametrize("service_name,expected_header,test_i</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC022].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:04:23</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>test_TC016_dashboard_patient_greeting</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="724c728b3a1a68b9276286209c33c7d5")&gt;
+    def test_TC016_dashboard_patient_greeting(driver):
+        """TC016: Patient dashboard greeting message and username rendering"""
+        dashb</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC016_dashboard_patient_greeting.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:04:37</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>test_TC017_last_diagnostic_card</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="279704dc4daad6b03f579f2efa507ba3")&gt;
+    def test_TC017_last_diagnostic_card(driver):
+        """TC017: Last diagnostic status card check"""
+        dashboard = login_and_get_dashboard</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC017_last_diagnostic_card.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:04:49</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>test_TC018_quick_services_presence</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="812a5297b4d0688a3b63f483157c83ab")&gt;
+    def test_TC018_quick_services_presence(driver):
+        """TC018: Quick services links presence verification"""
+        dashboard = login_and_g</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC018_quick_services_presence.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:05:08</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>test_TC019_navigation_bottom_bar_links</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="7e396889e5a8e218a38bac78879551ba")&gt;
+    def test_TC019_navigation_bottom_bar_links(driver):
+        """TC019: Navigation bottom bar links verification"""
+        dashboard = login_and</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC019_navigation_bottom_bar_links.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:05:34</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC020]</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="f97435015f90333b0946e0b69c08ba98")&gt;
+service_name = 'upload', expected_header = 'AI Lung Diagnosis'
+test_id = 'TC020'
+    @pytest.mark.parametrize("service_name,expected_header,test_id</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC020].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-07-17 12:05:52</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC021]</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="df6ece89376470411fc5b510a158c5e4")&gt;
+service_name = 'exercises', expected_header = 'Guided Exercises'
+test_id = 'TC021'
+    @pytest.mark.parametrize("service_name,expected_header,test_</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC021].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:23:44</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>test_TC016_dashboard_patient_greeting</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="32e7169d759c71908212ce63a8645275")&gt;
+    def test_TC016_dashboard_patient_greeting(driver):
+        """TC016: Patient dashboard greeting message and username rendering"""
+        dashb</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC016_dashboard_patient_greeting.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:24:11</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>test_TC017_last_diagnostic_card</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="2e993b5675333748227219595d8f9b21")&gt;
+    def test_TC017_last_diagnostic_card(driver):
+        """TC017: Last diagnostic status card check"""
+        dashboard = login_and_get_dashboard</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC017_last_diagnostic_card.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:24:28</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>test_TC018_quick_services_presence</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="0fb08380869808afc1aaeed40db2b178")&gt;
+    def test_TC018_quick_services_presence(driver):
+        """TC018: Quick services links presence verification"""
+        dashboard = login_and_g</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC018_quick_services_presence.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:24:47</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>test_TC019_navigation_bottom_bar_links</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="d5347c559179d155fb09e63c6d184a22")&gt;
+    def test_TC019_navigation_bottom_bar_links(driver):
+        """TC019: Navigation bottom bar links verification"""
+        dashboard = login_and</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC019_navigation_bottom_bar_links.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:25:06</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC020]</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="4bcfa3275b467d357d0257d47f852ec8")&gt;
+service_name = 'upload', expected_header = 'AI Lung Diagnosis'
+test_id = 'TC020'
+    @pytest.mark.parametrize("service_name,expected_header,test_id</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC020].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:25:25</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC021]</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="0fbc257420fec7848aac002c17c4c91c")&gt;
+service_name = 'exercises', expected_header = 'Guided Exercises'
+test_id = 'TC021'
+    @pytest.mark.parametrize("service_name,expected_header,test_</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC021].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:25:28</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>test_TC016_dashboard_patient_greeting</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="ec2ec0fcafee68cbbc9673f386bb4016")&gt;
+    def test_TC016_dashboard_patient_greeting(driver):
+        """TC016: Patient dashboard greeting message and username rendering"""
+        dashb</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC016_dashboard_patient_greeting.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:25:55</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC022]</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="e4c753e5af0fa88b874628e655061d87")&gt;
+service_name = 'medication', expected_header = 'Medication Log'
+test_id = 'TC022'
+    @pytest.mark.parametrize("service_name,expected_header,test_i</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC022].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:26:23</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>test_TC020_TC023_quick_links_navigation[TC023]</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="64f1260c936a5e004e7923e38846bb9e")&gt;
+service_name = 'hospitals', expected_header = 'Hospital Finder'
+test_id = 'TC023'
+    @pytest.mark.parametrize("service_name,expected_header,test_i</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC020_TC023_quick_links_navigation[TC023].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:26:55</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC024-Verify Doctor Dashboard stats tiles]</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:27:07</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC025-Verify Doctor today's consultation log table]</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:27:18</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC026-Add Patient Positive account creation]</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:27:39</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC027-Add Patient Duplicate email check]</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:27:51</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>test_TC001_successful_patient_login</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="cd484c094a8414eb78b33e1d7d4ad7b9")&gt;
+    def test_TC001_successful_patient_login(driver):
+        """TC001: Successful patient login with valid credentials"""
+        driver.get("http:</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC001_successful_patient_login.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:00</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC028-Add Patient Invalid email format check]</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:07</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC029-Add Patient Short password warning]</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:23</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC030-Add Patient Blank name validation]</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:30</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC031-Add Patient Blank email validation]</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:40</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC032-Add Patient Blank password validation]</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:52</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC033-Add Patient Login redirect link check]</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:28:57</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC034-Add Patient Onboarding loaders splash check]</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:29:02</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>test_dashboard_and_patient_additional_cases[TC035-Add Patient Onboarding skip bypass check]</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:29:22</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>test_TC046_navigate_to_review_center</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="af28d271caac4d0ea4d5a0fb260aec8a")&gt;
+    def test_TC046_navigate_to_review_center(driver):
+        """TC046: Doctor sidebar review center navigation tab click works"""
+        doctor_p</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC046_navigate_to_review_center.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:29:40</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>test_TC047_review_layout_headers</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="58aa192925c76a9976ed0e929b580aa6")&gt;
+    def test_TC047_review_layout_headers(driver):
+        """TC047: Verify review center layouts and title headings"""
+        doctor_page = login_</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC047_review_layout_headers.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:01</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>test_TC048_patient_scan_stats</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="a4c8fb184e9f54e99c759e2b9b9bb8d5")&gt;
+    def test_TC048_patient_scan_stats(driver):
+        """TC048: Check flagged patient details card contents"""
+        doctor_page = login_as_doct</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC048_patient_scan_stats.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:19</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>test_TC049_TC050_TC051_sign_off_scan</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="75075310babad344c2f19f6983d0ff03")&gt;
+    def test_TC049_TC050_TC051_sign_off_scan(driver):
+        """TC049, TC050, TC051: Sign off diagnostic lung scan and verify button states"""
+   </t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC049_TC050_TC051_sign_off_scan.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:38</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>test_TC052_sign_off_persistence</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="347edd7079aed4a63db2e0efcc15f62f")&gt;
+    def test_TC052_sign_off_persistence(driver):
+        """TC052: Sign-off remains persistent across browser reloads"""
+        doctor_page = logi</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC052_sign_off_persistence.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:42</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>test_doctor_portal_additional_cases[TC053-Verify doctor dashboard appointment stats auto update]</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:47</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>test_doctor_portal_additional_cases[TC054-Doctor telehealth video consult join call link routing]</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:30:53</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>test_doctor_portal_additional_cases[TC055-Verify doctor consultations video frame UI feeds overlays]</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:31:10</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>test_TC001_successful_patient_login</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="175e2333c2fbe6fb8b5738fb35ca9b3a")&gt;
+    def test_TC001_successful_patient_login(driver):
+        """TC001: Successful patient login with valid credentials"""
+        driver.get("http:</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC001_successful_patient_login.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:31:32</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>test_TC002_TC003_login_validation_errors[TC002]</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="1d470380da2bc430b8c15c0f02498e8c")&gt;
+email = 'invalidemail', password = 'password123'
+expected_error = 'Please enter a valid email address', test_id = 'TC002'
+    @pytest.mark.parametr</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC002_TC003_login_validation_errors[TC002].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:31:56</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>test_TC002_TC003_login_validation_errors[TC003]</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="bd5dab237d26837c86058914ef5822bf")&gt;
+email = 'patient@test.com', password = '123'
+expected_error = 'Password must be at least 6 characters', test_id = 'TC003'
+    @pytest.mark.parametr</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC002_TC003_login_validation_errors[TC003].png</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:32:14</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>test_TC004_TC005_empty_fields_validation</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="8ebb33d60b1e3d9bd458753c132de019")&gt;
+    def test_TC004_TC005_empty_fields_validation(driver):
+        """TC004 &amp; TC005: Form submission blocked for empty values"""
+        driver.get(</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC004_TC005_empty_fields_validation.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:32:36</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>test_TC006_incorrect_credentials_error</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="4793d80f43665c5495b03d3cfaa1f3ba")&gt;
+    def test_TC006_incorrect_credentials_error(driver):
+        """TC006: Patient login with incorrect password displays database error"""
+        </t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC006_incorrect_credentials_error.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:32:48</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>test_TC008_verify_login_ui_elements</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="9644bfd64ea6472a0705eb208919d2ef")&gt;
+    def test_TC008_verify_login_ui_elements(driver):
+        """TC008: Verify presence of logo and welcome header"""
+        driver.get("http://127</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC008_verify_login_ui_elements.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:33:04</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>test_TC009_verify_placeholder_texts</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="a1602efe1fd063a8955306edefd05131")&gt;
+    def test_TC009_verify_placeholder_texts(driver):
+        """TC009: Verify placeholder texts on inputs"""
+        driver.get("http://127.0.0.1:8</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC009_verify_placeholder_texts.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:33:23</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>test_TC010_verify_signup_navigation_link</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="ea5bc5eb07740c4e73b9591b71126fd8")&gt;
+    def test_TC010_verify_signup_navigation_link(driver):
+        """TC010: Verify navigation link to Registration page"""
+        driver.get("http</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC010_verify_signup_navigation_link.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:33:39</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>test_TC011_patient_logout_via_profile</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="0f283ceee07a2b0cd60b7b77585c63cd")&gt;
+    def test_TC011_patient_logout_via_profile(driver):
+        """TC011: Patient user logout via Profile tab redirects to Login"""
+        driver.g</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC011_patient_logout_via_profile.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:33:49</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>test_login_logout_additional_cases[TC007-Successful doctor login]</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:34:03</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>test_login_logout_additional_cases[TC012-Doctor user logout via Sidebar]</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:34:11</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>test_login_logout_additional_cases[TC013-Verify session cache is cleared on logout]</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:34:23</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>test_login_logout_additional_cases[TC014-Verify back button is blocked after logout]</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:34:37</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>test_login_logout_additional_cases[TC015-Verify logout button iconography]</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:34:55</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>test_TC086_TC087_TC088_TC089_book_telehealth</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="90e0979a333cba87374ae526abbdd5ac")&gt;
+    def test_TC086_TC087_TC088_TC089_book_telehealth(driver):
+        """TC086 to TC089: Select pulmonologist and schedule telehealth consultation </t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC086_TC087_TC088_TC089_book_telehealth.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:07</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>test_TC093_TC094_onboarding_swipe_navigation</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="c74bbe5a8b22ce4eed2a7a9039f652cc")&gt;
+    def test_TC093_TC094_onboarding_swipe_navigation(driver):
+        """TC093 &amp; TC094: Onboarding slider navigation next triggers screen swiping c</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC093_TC094_onboarding_swipe_navigation.png</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
ci: align jobs structure with main-ci-cd.yml workflow diagram
</commit_message>
<xml_diff>
--- a/selenium/reports/test_results.xlsx
+++ b/selenium/reports/test_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E62"/>
+  <dimension ref="A1:E114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2209,6 +2209,1444 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:26</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>test_TC096_TC097_session_handling_security</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="efa4552efa09dc56cc8915533a72afd1")&gt;
+    def test_TC096_TC097_session_handling_security(driver):
+        """TC096 &amp; TC097: Redirect non-authenticated users, and restore active cache se</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC096_TC097_session_handling_security.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:31</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC090-Verification of telehealth booking confirm notification Toast alert contents]</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:36</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC091-Pulmonologists directory consult scheduling back button click routing]</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:46</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC092-Doctor appointment consult video layout End call action confirmation popup]</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:51</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC095-Patient app notification logs clear all actions clicks verification]</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:35:59</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC098-Reload page validation ensures session data cache states persist correctly]</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:36:08</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC099-Resizing browser sizes adjusts patient portal grid layouts cleanly]</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:36:19</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC100-Validate browser console logs and verify no runtime console crash warnings]</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:36:28</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC101-Unit test FEV1 mathematical computations parsing logic returns values]</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:36:44</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC102-Unit test offline states properties fallbacks when database failed]</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:37:00</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC103-Unit test medications records checklists structures formats parser]</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:37:24</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC104-Unit test chats timestamp relative details calculations strings formats]</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:37:46</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC105-Unit test client side biometric encryption key signature checks values]</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:00</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC106-UI/UX Font style typography check for custom Google outfit formats]</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:04</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC107-UI/UX Contrast ratio accessibility compliance review checks rendering]</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:15</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC108-UI/UX Timer dynamic states frames animation updates loops smoothly]</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:28</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC109-UI/UX Mobile navigation layouts responsiveness adjustments verify sizes]</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:33</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>test_navigation_and_session_additional_cases[TC110-UI/UX Image alternative attributes verification checks rendering labels]</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:38:58</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>test_TC036_profile_update_fields</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="85dba4c7a7e744fa5cc5a0dc14c2521a")&gt;
+    def test_TC036_profile_update_fields(driver):
+        """TC036: Edit profile details (name and bio) and save successfully"""
+&gt;       profile_pa</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC036_profile_update_fields.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:39:21</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>test_TC037_profile_empty_name</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="77224fe35c7edb68705e0cb54cbda74f")&gt;
+    def test_TC037_profile_empty_name(driver):
+        """TC037: Profile validation warning displays on saving empty profile name"""
+&gt;       profil</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC037_profile_empty_name.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:39:39</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>test_TC039_toggle_biometrics</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="8ea85b85cf8516013589fb2c6eae2267")&gt;
+    def test_TC039_toggle_biometrics(driver):
+        """TC039: Toggle biometrics verification switch works"""
+&gt;       profile_page = login_and_nav</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC039_toggle_biometrics.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:39:44</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC038-Profile bio accepts maximum character limit constraints]</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:39:53</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC040-Profile avatar correctly reflects name initials placeholder]</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:05</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC041-Inputs pre-populated with current logged in credentials]</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:11</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC042-Update medication log checkboxes status]</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:17</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC043-Add new prescription medication log successfully]</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:23</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC044-Form validation on medication name blank input]</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:30</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>test_profile_form_additional_cases[TC045-Delete medication entry from log checklist]</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:40:53</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>test_TC076_reports_compiler_page_visible</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="0b4f5e5e3b3cfb11f84b4f52d2970f5b")&gt;
+    def test_TC076_reports_compiler_page_visible(driver):
+        """TC076: Generate PDF report compile page renders correctly"""
+&gt;       reports_p</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC076_reports_compiler_page_visible.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:41:36</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>test_TC077_default_reports_date_range</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="12f799a17f341b42a9072e83168cb120")&gt;
+    def test_TC077_default_reports_date_range(driver):
+        """TC077: Check start and end date default configurations load"""
+&gt;       reports_pa</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC077_default_reports_date_range.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:41:57</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>test_TC081_generate_pdf_report</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t xml:space="preserve">driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="1df1c8976793fe4651cb9d4b2d95570a")&gt;
+    def test_TC081_generate_pdf_report(driver):
+        """TC081: Compile report and verify print action behaves correctly"""
+&gt;       reports_page </t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC081_generate_pdf_report.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:15</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>test_TC082_report_back_button</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="94cf7ae1c9ae5e8c10c73d5c5c2ca028")&gt;
+    def test_TC082_report_back_button(driver):
+        """TC082: Clicks back button on reports page and returns back to dashboard home"""
+&gt;       r</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC082_report_back_button.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:21</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC078-Validation warnings displayed when start date input parameter blank]</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:27</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC079-Validation warnings displayed when end date input parameter blank]</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:34</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC080-Boundary checks block invalid date range input variables]</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:39</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC083-Historical scans results report list popup trigger]</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:45</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC084-Verify historical scans results report card header structures]</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:42:50</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>test_reports_additional_cases[TC085-Verify historical scan report modal is dismissed successfully]</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:43:02</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>test_app_load_and_login_detection</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:43:24</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>test_TC056_TC057_TC058_tab_switching_and_instructions</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="5db714c6a9dbb389c7784b5f8179f388")&gt;
+    def test_TC056_TC057_TC058_tab_switching_and_instructions(driver):
+        """TC056, TC057, TC058: Verify instructions display and upload/camer</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC056_TC057_TC058_tab_switching_and_instructions.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:43:44</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>test_TC059_file_upload_triggers_processing</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="c43812fae8f7542f73488750757c81d6")&gt;
+    def test_TC059_file_upload_triggers_processing(driver):
+        """TC059: Selecting a valid lung scan file successfully triggers AI analysis lo</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC059_file_upload_triggers_processing.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:02</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>test_TC060_TC061_camera_shutter_triggers_processing</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="8a3385d90067715380604220d2ecfc3c")&gt;
+    def test_TC060_TC061_camera_shutter_triggers_processing(driver):
+        """TC060, TC061: Capture scan report via simulated camera snaps correc</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC060_TC061_camera_shutter_triggers_processing.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:22</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>test_TC066_TC067_TC068_TC069_TC070_analysis_flow</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="41f776af48714f69725076736abe285e")&gt;
+    def test_TC066_TC067_TC068_TC069_TC070_analysis_flow(driver):
+        """TC066 to TC070: Complete AI diagnosis workflow, verify loader progress</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC066_TC067_TC068_TC069_TC070_analysis_flow.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:43</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>test_TC071_severity_status_badge</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>FAILED</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>driver = &lt;selenium.webdriver.chrome.webdriver.WebDriver (session="09de612d8b8152867d1b070548f4ec68")&gt;
+    def test_TC071_severity_status_badge(driver):
+        """TC071: Verify status colors badge tags represent severity scale indexes"""
+&gt;       upl</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>screenshots\test_TC071_severity_status_badge.png</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:48</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC062-Back button redirection returns to dashboard]</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:55</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC063-Boundary upload validation check on files over 10MB]</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:44:59</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC064-Validation formats check on unsupported files types]</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:45:05</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC065-Verify active optical line scanner animations visual status]</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:45:10</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC072-Check clinical recommendation list matches severity indexing criteria]</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:45:15</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC073-Verify lung volume FEV1 line analytical charts render canvases]</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:45:19</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC074-Verify Google/Leaflet API hospital layout map finders load]</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>2026-07-23 18:45:26</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>test_upload_and_ai_additional_cases[TC075-Locate search marker on entering nearest hospital locations query]</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>PASSED</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>